<commit_message>
v1.1.9: auto backfill BOM unit price (monthly weighted avg) and standard finished price (sum qty*price) after settlement; BOM ledger page
</commit_message>
<xml_diff>
--- a/sample_templates/BOM表.xlsx
+++ b/sample_templates/BOM表.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -605,32 +605,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -642,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -689,21 +663,42 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>5. 单价（子项物料的单价）、标准成品单价：仅存档，平台核算按实际投料×月末加权价。</t>
+          <t>5. 单价（子项物料的单价）、标准成品单价：**不用填**，系统在结算后自动回填：</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>6. 一个工单多子项就多行；项次按ERP原样填。</t>
+          <t xml:space="preserve">   子项单价 = 该子项物料本月月末加权平均价；</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">   标准成品单价 = 按工单汇总 Σ(子项用量 × 子项单价)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6. 一个工单多子项就多行；项次按ERP原样填。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>7. 表头行必须保留在第1行；示例行（黄底）上传前请删除。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8. 导入后可到「BOM表台账」查看系统回填的单价。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.1.10: BOM template add serial no. column as first column (ignored on import); fix line_no alias
</commit_message>
<xml_diff>
--- a/sample_templates/BOM表.xlsx
+++ b/sample_templates/BOM表.xlsx
@@ -434,177 +434,207 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>工单编号</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>物料编号</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>物料名称</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>项次</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>子项物料编号</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>子项物料名称</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>子项用量:分子</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>子项用量:分母</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>单位名称</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>单价（子项物料的单价）</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>标准成品单价</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>BC-16.0026CS-20260720</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>BC-16.0026</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>烟台对位芳纶粗纱</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>R11.125</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>对位芳纶长丝</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="H2" s="2" t="n">
         <v>1000</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
-        <v>120.5</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>125</v>
-      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>11.21-20260720</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>11.21</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>对位芳纶纱线</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>BC-16.0026</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>烟台对位芳纶粗纱</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>105</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="I3" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
-        <v>130</v>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -616,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -649,56 +679,63 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>3. 必填列：工单编号、子项物料编号；其余列可留空。</t>
+          <t>3. 序号：ERP导出的行序号，仅存档，平台不读取；可留空。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>4. 子项用量:分子 / 子项用量:分母：子项用量以分数表示（如 105/100 = 生产1单位父项消耗1.05子项）。</t>
+          <t>4. 必填列：工单编号、子项物料编号；其余列可留空。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>5. 单价（子项物料的单价）、标准成品单价：**不用填**，系统在结算后自动回填：</t>
+          <t>5. 子项用量:分子 / 子项用量:分母：子项用量以分数表示（如 105/100 = 生产1单位父项消耗1.05子项）。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">   子项单价 = 该子项物料本月月末加权平均价；</t>
+          <t>6. 单价（子项物料的单价）、标准成品单价：**不用填**，系统在结算后自动回填：</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">   子项单价 = 该子项物料本月月末加权平均价；</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">   标准成品单价 = 按工单汇总 Σ(子项用量 × 子项单价)。</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>6. 一个工单多子项就多行；项次按ERP原样填。</t>
-        </is>
-      </c>
-    </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>7. 表头行必须保留在第1行；示例行（黄底）上传前请删除。</t>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>7. 一个工单多子项就多行；项次按ERP原样填。</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>8. 导入后可到「BOM表台账」查看系统回填的单价。</t>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>8. 表头行必须保留在第1行；示例行（黄底）上传前请删除。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>9. 导入后可到「BOM表台账」查看系统回填的单价。</t>
         </is>
       </c>
     </row>

</xml_diff>